<commit_message>
Add digital membership card with QR verification
- Membership numbers are issued on approval as TC-YY-RRR-NNNNNN-C
  (year, region, yearly sequence, Luhn check digit); never reused.
- Member card page (/app/card) with server-rendered QR code, print/PDF,
  accurate status, and "get a new QR code" for lost or shared cards.
- Public /verify/{token} and /verify (by number): status and short name
  for everyone, full details for officers with Verify Membership;
  rate-limited, noindex, every check logged in membership_verifications.
- API: membership/card, membership/card/reissue, membership/verify.
- Adds bacon/bacon-qr-code for QR generation.
- Kiswahili translations, README, decisions D-03/D-13 and RTM updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RYPH4vgdjTcpHQVRwFcZuL
</commit_message>
<xml_diff>
--- a/docs/Requirements-Traceability-Matrix.xlsx
+++ b/docs/Requirements-Traceability-Matrix.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document Release 1: roles, sign-in security, new screens
- README: new member and admin URLs, roles table (Super Admin,
  Coordinator, Patron, nationwide officer), staff SMS sign-in and token
  expiry, post-pull seed steps.
- Decisions D-08, D-09 and D-12 recorded as implemented, pending
  confirmation; all 25 Release 1 requirements marked Done in the RTM.
- Screenshots of the new screens.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RYPH4vgdjTcpHQVRwFcZuL
</commit_message>
<xml_diff>
--- a/docs/Requirements-Traceability-Matrix.xlsx
+++ b/docs/Requirements-Traceability-Matrix.xlsx
@@ -966,7 +966,7 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="S85" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="S86" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8440,7 +8440,7 @@
       </c>
       <c r="S90" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8527,7 +8527,7 @@
       </c>
       <c r="S91" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Release 3: navigation, Kiswahili translations, docs, RTM and screenshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RYPH4vgdjTcpHQVRwFcZuL
</commit_message>
<xml_diff>
--- a/docs/Requirements-Traceability-Matrix.xlsx
+++ b/docs/Requirements-Traceability-Matrix.xlsx
@@ -4932,7 +4932,7 @@
       </c>
       <c r="S50" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="S51" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5193,7 +5193,7 @@
       </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5367,7 +5367,7 @@
       </c>
       <c r="S55" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -5541,7 +5541,7 @@
       </c>
       <c r="S57" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7301,7 @@
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7388,7 +7388,7 @@
       </c>
       <c r="S78" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7475,7 +7475,7 @@
       </c>
       <c r="S79" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7562,7 +7562,7 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7736,7 +7736,7 @@
       </c>
       <c r="S82" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7823,7 +7823,7 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7910,7 +7910,7 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="S87" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8266,7 +8266,7 @@
       </c>
       <c r="S88" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8614,7 +8614,7 @@
       </c>
       <c r="S92" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="S93" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8875,7 +8875,7 @@
       </c>
       <c r="S95" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add R4/R5 navigation, default spaces seeder and documentation
- Navigation for community, Ask TRA, competitions, rewards, alumni and mentorship
- CommunityAndRewardsSeeder: national and club spaces, starter rewards
- README, API spec, decisions register and RTM updated for Releases 4 and 5

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RYPH4vgdjTcpHQVRwFcZuL
</commit_message>
<xml_diff>
--- a/docs/Requirements-Traceability-Matrix.xlsx
+++ b/docs/Requirements-Traceability-Matrix.xlsx
@@ -3354,7 +3354,7 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3441,7 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="S34" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="S35" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="S36" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3793,7 @@
       </c>
       <c r="S37" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="S38" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4054,7 @@
       </c>
       <c r="S40" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="S41" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4228,7 @@
       </c>
       <c r="S42" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="S46" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="S48" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="S68" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6593,7 +6593,7 @@
       </c>
       <c r="S69" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6680,7 +6680,7 @@
       </c>
       <c r="S70" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6767,7 +6767,7 @@
       </c>
       <c r="S71" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6854,7 +6854,7 @@
       </c>
       <c r="S72" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -6945,7 +6945,7 @@
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="S74" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="S75" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="S76" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="S96" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9049,7 +9049,7 @@
       </c>
       <c r="S97" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="S98" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="S99" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9314,7 +9314,7 @@
       </c>
       <c r="S100" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9405,7 @@
       </c>
       <c r="S101" s="2" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>